<commit_message>
feat: update data file with new player statistics and performance metrics
</commit_message>
<xml_diff>
--- a/data/內運週二團第二季試辦比賽.xlsx
+++ b/data/內運週二團第二季試辦比賽.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\n1025\Desktop\NBA選秀\NBA-\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA514AEF-1412-44DC-8743-A29B19C0EA00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CBEF306-FA54-4C30-8EDF-C7CFA235D666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NEUTEC 組隊報名區" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="35">
   <si>
     <t>*預計組二隊，一隊最少 5 人，最多 8 人，方便累的時侯可以換人
 *6/23 第一輪四隊輪打，一場 12 分鐘，如果報名完只有三隊會再調整比賽時長
@@ -122,6 +122,26 @@
     <t>Paul(DI)</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
+  <si>
+    <t>鋒線</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>18:00 ~ 19:00</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>James</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>後衛</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Kai</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -130,7 +150,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="mm/dd"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -197,6 +217,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="微軟正黑體"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -218,7 +245,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -247,6 +274,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -465,9 +494,10 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="21.42578125" customWidth="1"/>
     <col min="3" max="3" width="22.28515625" customWidth="1"/>
     <col min="4" max="4" width="18.42578125" customWidth="1"/>
     <col min="5" max="5" width="7.42578125" bestFit="1" customWidth="1"/>
@@ -585,8 +615,8 @@
       <c r="B8" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>14</v>
+      <c r="C8" s="15" t="s">
+        <v>31</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>7</v>
@@ -768,12 +798,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="5" t="s">
-        <v>11</v>
+      <c r="B19" s="14" t="s">
+        <v>33</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>7</v>
@@ -786,12 +816,12 @@
       </c>
       <c r="F19" s="1"/>
     </row>
-    <row r="20" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>9</v>
+      <c r="B20" s="14" t="s">
+        <v>30</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>7</v>
@@ -803,6 +833,40 @@
         <v>3</v>
       </c>
       <c r="F20" s="1"/>
+    </row>
+    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" s="6">
+        <v>46196</v>
+      </c>
+      <c r="E21" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="6">
+        <v>46196</v>
+      </c>
+      <c r="E22" s="1">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -810,13 +874,13 @@
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B4:B20" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B4:B22" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"後衛,鋒線,中鋒"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C4:C20" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C4:C22" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"全程,18:00 ~ 19:00,19:00 ~ 20:00"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D4:D20" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D4:D22" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"全程,06/23,06/30"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>